<commit_message>
doc(jdt) Mise à jour JdT
</commit_message>
<xml_diff>
--- a/Jdt-P_FUN.xlsx
+++ b/Jdt-P_FUN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okkeserdem/Documents/ETML/Projets/P_Fun/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9FF11DA-9BC6-B843-AED9-E91FBF68EE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F94CD5-0306-CC4F-8125-4B77ECF725D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
   <si>
     <t>Semaine</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>Changement US : Affichage interface graphique</t>
+  </si>
+  <si>
+    <t>Absent</t>
+  </si>
+  <si>
+    <t>Absent de 8h à 10h</t>
   </si>
 </sst>
 </file>
@@ -159,6 +165,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -240,12 +247,6 @@
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -256,6 +257,12 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -271,14 +278,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau1" displayName="Tableau1" ref="A1:E39" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau1" displayName="Tableau1" ref="A1:E39" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:E39" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Semaine" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Durée" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tâche" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Remarque" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Semaine" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Durée" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tâche" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Remarque" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1072,14 +1079,16 @@
         <v>14.09</v>
       </c>
       <c r="C32" s="4">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32" s="6"/>
-    </row>
-    <row r="33" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="4">
         <v>4</v>
       </c>
@@ -1087,16 +1096,14 @@
         <v>14.09</v>
       </c>
       <c r="C33" s="4">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="E33" s="6"/>
+    </row>
+    <row r="34" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A34" s="4">
         <v>4</v>
       </c>
@@ -1104,12 +1111,14 @@
         <v>14.09</v>
       </c>
       <c r="C34" s="4">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E34" s="6"/>
+        <v>35</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="4">
@@ -1119,10 +1128,10 @@
         <v>14.09</v>
       </c>
       <c r="C35" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E35" s="6"/>
     </row>
@@ -1142,10 +1151,18 @@
       <c r="E36" s="6"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
+      <c r="A37" s="4">
+        <v>4</v>
+      </c>
+      <c r="B37" s="4">
+        <v>14.09</v>
+      </c>
+      <c r="C37" s="4">
+        <v>15</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="E37" s="6"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1165,7 +1182,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="88" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="93" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
feat(tests) Ajout test unitaire
</commit_message>
<xml_diff>
--- a/Jdt-P_FUN.xlsx
+++ b/Jdt-P_FUN.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okkeserdem/Documents/ETML/Projets/P_FUN/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B57C584-207B-0642-842A-1464B48BD21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -18,12 +12,12 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$53</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="69">
   <si>
     <t>Semaine</t>
   </si>
@@ -115,19 +109,25 @@
     <t>Ajoute limite de zoom</t>
   </si>
   <si>
+    <t>Création Parser pour Weather</t>
+  </si>
+  <si>
+    <t>Ajout classe Weather</t>
+  </si>
+  <si>
+    <t>Créations données fictives</t>
+  </si>
+  <si>
+    <t>Modification du GUI</t>
+  </si>
+  <si>
     <t>Ajout de la classe DataSeries au project</t>
   </si>
   <si>
-    <t>Ajout classe Weather</t>
-  </si>
-  <si>
-    <t>Créations données fictives</t>
-  </si>
-  <si>
-    <t>Création Parser pour Weather</t>
-  </si>
-  <si>
-    <t>Modification du GUI</t>
+    <t>Absent</t>
+  </si>
+  <si>
+    <t>Absent de 8h à 10h</t>
   </si>
   <si>
     <t>Mise à jour du repo GIT</t>
@@ -142,12 +142,6 @@
     <t>Changement US : Affichage interface graphique</t>
   </si>
   <si>
-    <t>Absent</t>
-  </si>
-  <si>
-    <t>Absent de 8h à 10h</t>
-  </si>
-  <si>
     <t>Congé</t>
   </si>
   <si>
@@ -178,12 +172,12 @@
     <t>Amélioration des exports</t>
   </si>
   <si>
+    <t>Ajout de commentaires</t>
+  </si>
+  <si>
     <t>Discution avec le prof</t>
   </si>
   <si>
-    <t>Ajout de commentaires</t>
-  </si>
-  <si>
     <t>Fonction d'actualisation</t>
   </si>
   <si>
@@ -200,13 +194,43 @@
   </si>
   <si>
     <t>J'ai pris du temps pour améliorer le code, notamment enlever les 'var' pour mettre leur vraie types</t>
+  </si>
+  <si>
+    <t>Refactor code</t>
+  </si>
+  <si>
+    <t>Suppression de foreach dans la fonction reload data</t>
+  </si>
+  <si>
+    <t>Refactor import click func et refresh plot</t>
+  </si>
+  <si>
+    <t>amélioration des select des fichiers</t>
+  </si>
+  <si>
+    <t>Selection de csv uniquement</t>
+  </si>
+  <si>
+    <t>Export PNG à taille de graphique</t>
+  </si>
+  <si>
+    <t>Exporter uniquement les cases des villes cochées</t>
+  </si>
+  <si>
+    <t>Ajout filtre par date</t>
+  </si>
+  <si>
+    <t>Correction de l'UI</t>
+  </si>
+  <si>
+    <t>Utilisation de l'IA pour regler les probleme de responsive et de scroll bar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -222,12 +246,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
@@ -240,11 +258,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="9.9978637043366805E-2"/>
+      <patternFill patternType="gray125">
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -252,6 +266,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.1"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -310,7 +330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -318,7 +338,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -327,22 +347,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -351,60 +371,132 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tableau1" displayName="Tableau1" ref="A1:E59" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E59" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:E74" totalsRowShown="0">
+  <autoFilter ref="A1:E74"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Semaine" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Durée" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tâche" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Remarque" dataDxfId="0"/>
+    <tableColumn id="1" name="Semaine"/>
+    <tableColumn id="2" name="Date"/>
+    <tableColumn id="3" name="Durée"/>
+    <tableColumn id="4" name="Tâche"/>
+    <tableColumn id="5" name="Remarque"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -413,12 +505,12 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Thème Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -451,9 +543,9 @@
         <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Thème Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -505,7 +597,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -557,85 +649,36 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Craft">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -646,13 +689,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -660,86 +697,35 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E74"/>
+  <sheetFormatPr defaultColWidth="11.421875" defaultRowHeight="16" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="12" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="45" style="2" customWidth="1"/>
-    <col min="5" max="5" width="48.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.00390625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="12.421875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="15.00390625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="54.140625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="48.421875" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -749,14 +735,14 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="45" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" ht="16.5">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -769,9 +755,9 @@
       <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="13"/>
-    </row>
-    <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E2" s="8"/>
+    </row>
+    <row r="3" ht="16.5">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -784,11 +770,11 @@
       <c r="D3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" ht="16.5">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -801,9 +787,9 @@
       <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E4" s="8"/>
+    </row>
+    <row r="5" ht="16.5">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -816,9 +802,9 @@
       <c r="D5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="13"/>
-    </row>
-    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E5" s="8"/>
+    </row>
+    <row r="6" ht="16.5">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -831,18 +817,18 @@
       <c r="D6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" ht="16.5">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="14"/>
-    </row>
-    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E7" s="46"/>
+    </row>
+    <row r="8" ht="16.5">
       <c r="A8" s="4">
         <v>2</v>
       </c>
@@ -855,11 +841,11 @@
       <c r="D8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" ht="16.5">
       <c r="A9" s="4">
         <v>2</v>
       </c>
@@ -872,11 +858,11 @@
       <c r="D9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" ht="16.5">
       <c r="A10" s="4">
         <v>2</v>
       </c>
@@ -889,11 +875,11 @@
       <c r="D10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" ht="16.5">
       <c r="A11" s="4">
         <v>2</v>
       </c>
@@ -906,11 +892,11 @@
       <c r="D11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" ht="16.5">
       <c r="A12" s="4">
         <v>2</v>
       </c>
@@ -923,11 +909,11 @@
       <c r="D12" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" ht="16.5">
       <c r="A13" s="4">
         <v>2</v>
       </c>
@@ -940,9 +926,9 @@
       <c r="D13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="13"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" ht="16.5">
       <c r="A14" s="4">
         <v>2</v>
       </c>
@@ -955,9 +941,9 @@
       <c r="D14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="13"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E14" s="8"/>
+    </row>
+    <row r="15" ht="16.5">
       <c r="A15" s="4">
         <v>2</v>
       </c>
@@ -970,9 +956,9 @@
       <c r="D15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="13"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E15" s="8"/>
+    </row>
+    <row r="16" ht="16.5">
       <c r="A16" s="4">
         <v>2</v>
       </c>
@@ -985,16 +971,16 @@
       <c r="D16" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="13"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" ht="16.5">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="14"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E17" s="46"/>
+    </row>
+    <row r="18" ht="16.5">
       <c r="A18" s="4">
         <v>3</v>
       </c>
@@ -1007,9 +993,9 @@
       <c r="D18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="13"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E18" s="8"/>
+    </row>
+    <row r="19" ht="16.5">
       <c r="A19" s="4">
         <v>3</v>
       </c>
@@ -1022,9 +1008,9 @@
       <c r="D19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="13"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E19" s="8"/>
+    </row>
+    <row r="20" ht="16.5">
       <c r="A20" s="4">
         <v>3</v>
       </c>
@@ -1037,9 +1023,9 @@
       <c r="D20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="13"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" ht="16.5">
       <c r="A21" s="4">
         <v>3</v>
       </c>
@@ -1052,9 +1038,9 @@
       <c r="D21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="13"/>
-    </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" ht="33.75">
       <c r="A22" s="4">
         <v>3</v>
       </c>
@@ -1067,11 +1053,11 @@
       <c r="D22" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" ht="16.5">
       <c r="A23" s="4">
         <v>3</v>
       </c>
@@ -1084,9 +1070,9 @@
       <c r="D23" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E23" s="13"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" ht="16.5">
       <c r="A24" s="4">
         <v>3</v>
       </c>
@@ -1099,9 +1085,9 @@
       <c r="D24" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="13"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" ht="16.5">
       <c r="A25" s="4">
         <v>3</v>
       </c>
@@ -1112,11 +1098,11 @@
         <v>25</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" s="13"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" ht="16.5">
       <c r="A26" s="4">
         <v>3</v>
       </c>
@@ -1129,9 +1115,9 @@
       <c r="D26" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="13"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E26" s="8"/>
+    </row>
+    <row r="27" ht="16.5">
       <c r="A27" s="4">
         <v>3</v>
       </c>
@@ -1144,16 +1130,16 @@
       <c r="D27" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="13"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E27" s="8"/>
+    </row>
+    <row r="28" ht="16.5">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
-      <c r="E28" s="14"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E28" s="46"/>
+    </row>
+    <row r="29" ht="16.5">
       <c r="A29" s="4">
         <v>3</v>
       </c>
@@ -1164,11 +1150,11 @@
         <v>10</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E29" s="13"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+      <c r="E29" s="8"/>
+    </row>
+    <row r="30" ht="16.5">
       <c r="A30" s="4">
         <v>3</v>
       </c>
@@ -1179,18 +1165,18 @@
         <v>10</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30" s="13"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+      <c r="E30" s="8"/>
+    </row>
+    <row r="31" ht="16.5">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="7"/>
-      <c r="E31" s="14"/>
-    </row>
-    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E31" s="46"/>
+    </row>
+    <row r="32" ht="16.5">
       <c r="A32" s="4">
         <v>4</v>
       </c>
@@ -1201,13 +1187,13 @@
         <v>90</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" ht="16.5">
       <c r="A33" s="4">
         <v>4</v>
       </c>
@@ -1220,9 +1206,9 @@
       <c r="D33" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E33" s="13"/>
-    </row>
-    <row r="34" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="E33" s="8"/>
+    </row>
+    <row r="34" ht="48">
       <c r="A34" s="4">
         <v>4</v>
       </c>
@@ -1233,13 +1219,13 @@
         <v>40</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" ht="16.5">
       <c r="A35" s="4">
         <v>4</v>
       </c>
@@ -1250,11 +1236,11 @@
         <v>10</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E35" s="13"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+      <c r="E35" s="8"/>
+    </row>
+    <row r="36" ht="16.5">
       <c r="A36" s="4">
         <v>4</v>
       </c>
@@ -1265,11 +1251,11 @@
         <v>15</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E36" s="13"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+      <c r="E36" s="8"/>
+    </row>
+    <row r="37" ht="16.5">
       <c r="A37" s="4">
         <v>4</v>
       </c>
@@ -1280,18 +1266,18 @@
         <v>15</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E37" s="13"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+      <c r="E37" s="8"/>
+    </row>
+    <row r="38" ht="16.5">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
       <c r="D38" s="7"/>
-      <c r="E38" s="14"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E38" s="46"/>
+    </row>
+    <row r="39" ht="16.5">
       <c r="A39" s="4">
         <v>5</v>
       </c>
@@ -1302,16 +1288,16 @@
       <c r="D39" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E39" s="13"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E39" s="8"/>
+    </row>
+    <row r="40" ht="16.5">
       <c r="A40" s="9"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
       <c r="D40" s="11"/>
-      <c r="E40" s="15"/>
-    </row>
-    <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E40" s="48"/>
+    </row>
+    <row r="41" ht="16.5">
       <c r="A41" s="4">
         <v>6</v>
       </c>
@@ -1320,13 +1306,13 @@
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E41" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E41" s="8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" ht="33.75">
       <c r="A42" s="4">
         <v>6</v>
       </c>
@@ -1339,11 +1325,11 @@
       <c r="D42" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E42" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" ht="16.5">
       <c r="A43" s="4">
         <v>6</v>
       </c>
@@ -1356,16 +1342,16 @@
       <c r="D43" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E43" s="13"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E43" s="8"/>
+    </row>
+    <row r="44" ht="16.5">
       <c r="A44" s="9"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
-      <c r="E44" s="15"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E44" s="48"/>
+    </row>
+    <row r="45" ht="16.5">
       <c r="A45" s="4">
         <v>7</v>
       </c>
@@ -1378,9 +1364,9 @@
       <c r="D45" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E45" s="13"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" ht="16.5">
       <c r="A46" s="4">
         <v>7</v>
       </c>
@@ -1393,9 +1379,9 @@
       <c r="D46" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E46" s="13"/>
-    </row>
-    <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="E46" s="8"/>
+    </row>
+    <row r="47" ht="16.5">
       <c r="A47" s="4">
         <v>7</v>
       </c>
@@ -1408,11 +1394,11 @@
       <c r="D47" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="E47" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" ht="16.5">
       <c r="A48" s="4">
         <v>7</v>
       </c>
@@ -1425,9 +1411,9 @@
       <c r="D48" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E48" s="13"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" ht="16.5">
       <c r="A49" s="4">
         <v>7</v>
       </c>
@@ -1440,9 +1426,9 @@
       <c r="D49" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E49" s="13"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" ht="16.5">
       <c r="A50" s="4">
         <v>7</v>
       </c>
@@ -1453,11 +1439,11 @@
         <v>15</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E50" s="13"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="E50" s="8"/>
+    </row>
+    <row r="51" ht="16.5">
       <c r="A51" s="4">
         <v>7</v>
       </c>
@@ -1468,18 +1454,18 @@
         <v>25</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E51" s="13"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+      <c r="E51" s="8"/>
+    </row>
+    <row r="52" ht="16.5">
       <c r="A52" s="9"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="11"/>
-      <c r="E52" s="15"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E52" s="48"/>
+    </row>
+    <row r="53" ht="16.5">
       <c r="A53" s="4">
         <v>8</v>
       </c>
@@ -1492,9 +1478,9 @@
       <c r="D53" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E53" s="13"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E53" s="8"/>
+    </row>
+    <row r="54" ht="16.5">
       <c r="A54" s="4">
         <v>8</v>
       </c>
@@ -1507,9 +1493,9 @@
       <c r="D54" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E54" s="13"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E54" s="8"/>
+    </row>
+    <row r="55" ht="16.5">
       <c r="A55" s="4">
         <v>8</v>
       </c>
@@ -1522,9 +1508,9 @@
       <c r="D55" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E55" s="13"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E55" s="8"/>
+    </row>
+    <row r="56" ht="16.5">
       <c r="A56" s="4">
         <v>8</v>
       </c>
@@ -1537,9 +1523,9 @@
       <c r="D56" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E56" s="13"/>
-    </row>
-    <row r="57" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="E56" s="8"/>
+    </row>
+    <row r="57" ht="48">
       <c r="A57" s="4">
         <v>8</v>
       </c>
@@ -1552,28 +1538,173 @@
       <c r="D57" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E57" s="13" t="s">
+      <c r="E57" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="13"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="13"/>
+    <row r="58" ht="33.75">
+      <c r="A58" s="4">
+        <v>8</v>
+      </c>
+      <c r="B58" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C58" s="4">
+        <v>15</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" ht="16.5">
+      <c r="A59" s="4">
+        <v>8</v>
+      </c>
+      <c r="B59" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C59" s="4">
+        <v>15</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="60" ht="16.5">
+      <c r="A60" s="4">
+        <v>8</v>
+      </c>
+      <c r="B60" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C60" s="4">
+        <v>10</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="61" ht="16.5">
+      <c r="A61" s="4">
+        <v>8</v>
+      </c>
+      <c r="B61" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C61" s="4">
+        <v>10</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E61" s="8"/>
+    </row>
+    <row r="62" ht="16.5">
+      <c r="A62" s="4">
+        <v>8</v>
+      </c>
+      <c r="B62" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C62" s="4">
+        <v>10</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5">
+      <c r="A63" s="4">
+        <v>8</v>
+      </c>
+      <c r="B63" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C63" s="4">
+        <v>10</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="64" ht="33.75">
+      <c r="A64" s="4">
+        <v>8</v>
+      </c>
+      <c r="B64" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C64" s="4">
+        <v>10</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="65" ht="16.5">
+      <c r="A65" s="4">
+        <v>8</v>
+      </c>
+      <c r="B65" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C65" s="4"/>
+      <c r="D65" s="5"/>
+    </row>
+    <row r="66" ht="16.5">
+      <c r="A66" s="4">
+        <v>8</v>
+      </c>
+      <c r="B66" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C66" s="4"/>
+      <c r="D66" s="5"/>
+    </row>
+    <row r="67" ht="16.5">
+      <c r="A67" s="4">
+        <v>8</v>
+      </c>
+      <c r="B67" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="5"/>
+    </row>
+    <row r="68" ht="16.5">
+      <c r="A68" s="4">
+        <v>8</v>
+      </c>
+      <c r="B68" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="5"/>
+    </row>
+    <row r="69" ht="16.5"/>
+    <row r="70" ht="16.5"/>
+    <row r="71" ht="16.5"/>
+    <row r="72" ht="16.5"/>
+    <row r="73" ht="16.5"/>
+    <row r="74" ht="16.5">
+      <c r="A74" s="4"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="8"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="93" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
+  <pageSetup paperSize="9" scale="93" fitToWidth="1" fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
ajout de data dans le repo
</commit_message>
<xml_diff>
--- a/Jdt-P_FUN.xlsx
+++ b/Jdt-P_FUN.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="73">
   <si>
     <t>Semaine</t>
   </si>
@@ -224,6 +224,18 @@
   </si>
   <si>
     <t>Utilisation de l'IA pour regler les probleme de responsive et de scroll bar</t>
+  </si>
+  <si>
+    <t>Affichage de message a l'ecran</t>
+  </si>
+  <si>
+    <t>Ajout test unitaire</t>
+  </si>
+  <si>
+    <t>Ajout extension</t>
+  </si>
+  <si>
+    <t>Ajout des data réeles</t>
   </si>
 </sst>
 </file>
@@ -1657,8 +1669,12 @@
       <c r="B65" s="12">
         <v>46325</v>
       </c>
-      <c r="C65" s="4"/>
-      <c r="D65" s="5"/>
+      <c r="C65" s="4">
+        <v>5</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="66" ht="16.5">
       <c r="A66" s="4">
@@ -1667,8 +1683,12 @@
       <c r="B66" s="12">
         <v>46325</v>
       </c>
-      <c r="C66" s="4"/>
-      <c r="D66" s="5"/>
+      <c r="C66" s="4">
+        <v>20</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="67" ht="16.5">
       <c r="A67" s="4">
@@ -1677,8 +1697,12 @@
       <c r="B67" s="12">
         <v>46325</v>
       </c>
-      <c r="C67" s="4"/>
-      <c r="D67" s="5"/>
+      <c r="C67" s="4">
+        <v>10</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="68" ht="16.5">
       <c r="A68" s="4">
@@ -1687,8 +1711,12 @@
       <c r="B68" s="12">
         <v>46325</v>
       </c>
-      <c r="C68" s="4"/>
-      <c r="D68" s="5"/>
+      <c r="C68" s="4">
+        <v>5</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="69" ht="16.5"/>
     <row r="70" ht="16.5"/>

</xml_diff>

<commit_message>
doc(jdt, readme) Maj des docs
</commit_message>
<xml_diff>
--- a/Jdt-P_FUN.xlsx
+++ b/Jdt-P_FUN.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="74">
   <si>
     <t>Semaine</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Ajout des data réeles</t>
+  </si>
+  <si>
+    <t>Finalistation rapport</t>
   </si>
 </sst>
 </file>
@@ -501,8 +504,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:E74" totalsRowShown="0">
-  <autoFilter ref="A1:E74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:E70" totalsRowShown="0">
+  <autoFilter ref="A1:E70"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Semaine"/>
     <tableColumn id="2" name="Date"/>
@@ -727,7 +730,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr defaultColWidth="11.421875" defaultRowHeight="16" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.00390625" style="4" customWidth="1"/>
@@ -1718,17 +1721,26 @@
         <v>72</v>
       </c>
     </row>
-    <row r="69" ht="16.5"/>
-    <row r="70" ht="16.5"/>
-    <row r="71" ht="16.5"/>
-    <row r="72" ht="16.5"/>
-    <row r="73" ht="16.5"/>
-    <row r="74" ht="16.5">
-      <c r="A74" s="4"/>
-      <c r="B74" s="4"/>
-      <c r="C74" s="4"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="8"/>
+    <row r="69" ht="16.5">
+      <c r="A69" s="4">
+        <v>8</v>
+      </c>
+      <c r="B69" s="12">
+        <v>46325</v>
+      </c>
+      <c r="C69" s="4">
+        <v>40</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="70" ht="16.5">
+      <c r="A70" s="4"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>

</xml_diff>